<commit_message>
Update the resync data code
</commit_message>
<xml_diff>
--- a/public/data/travel_north_bengal.xlsx
+++ b/public/data/travel_north_bengal.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="111">
   <si>
     <t xml:space="preserve">RailStation</t>
   </si>
@@ -305,6 +305,54 @@
   </si>
   <si>
     <t xml:space="preserve">26.1026,87.9485</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madaripur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.305524, 88.260835</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chopra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.380096, 88.312805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binnaguri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.657023, 88.416647</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gajoldoba View point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.750822, 88.585768</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dakshin Haskhali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.743245, 88.659656</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dhantala Market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.680222, 88.732484</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lataguri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.705837, 88.768500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gorumara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.758572, 88.786466</t>
   </si>
 </sst>
 </file>
@@ -392,7 +440,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -410,6 +458,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -536,7 +592,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.82"/>
@@ -591,9 +647,12 @@
       <c r="C3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="1" t="str">
+      <c r="D3" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="n">
         <f aca="false">IFERROR(C3/(D3/60),"")</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>11</v>
@@ -609,9 +668,12 @@
       <c r="C4" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="E4" s="1" t="str">
+      <c r="D4" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1" t="n">
         <f aca="false">IFERROR(C4/(D4/60),"")</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>14</v>
@@ -863,6 +925,9 @@
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
         <v>42</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <v>330</v>
       </c>
       <c r="E17" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C16/(D16/60),2),"")</f>
@@ -898,6 +963,9 @@
       <c r="B19" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="D19" s="0" t="n">
+        <v>340</v>
+      </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4" t="s">
         <v>48</v>
@@ -949,6 +1017,9 @@
       <c r="B22" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="D22" s="0" t="n">
+        <v>400</v>
+      </c>
       <c r="E22" s="1"/>
       <c r="F22" s="4" t="s">
         <v>56</v>
@@ -1105,6 +1176,16 @@
       <c r="B31" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="C31" s="1" t="n">
+        <v>426</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <v>515</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C31/(D31/60),2),"")</f>
+        <v>49.63</v>
+      </c>
       <c r="F31" s="4" t="s">
         <v>74</v>
       </c>
@@ -1131,9 +1212,12 @@
       <c r="B33" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E33" s="1" t="str">
+      <c r="D33" s="0" t="n">
+        <v>523</v>
+      </c>
+      <c r="E33" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C33/(D33/60),2),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>78</v>
@@ -1197,9 +1281,12 @@
       <c r="B37" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E37" s="1" t="str">
+      <c r="D37" s="0" t="n">
+        <v>548</v>
+      </c>
+      <c r="E37" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C37/(D37/60),2),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>86</v>
@@ -1209,9 +1296,12 @@
       <c r="B38" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="1" t="str">
+      <c r="D38" s="0" t="n">
+        <v>550</v>
+      </c>
+      <c r="E38" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C38/(D38/60),2),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>88</v>
@@ -1261,38 +1351,161 @@
         <v>481</v>
       </c>
       <c r="D41" s="1" t="n">
-        <v>581</v>
+        <v>600</v>
       </c>
       <c r="E41" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C41/(D41/60),2),"")</f>
-        <v>49.67</v>
+        <v>48.1</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E42" s="1" t="str">
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>523</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <v>653</v>
+      </c>
+      <c r="E42" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C42/(D42/60),2),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E43" s="1" t="str">
+        <v>48.06</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C43" s="1" t="n">
+        <v>533</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <v>666</v>
+      </c>
+      <c r="E43" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C43/(D43/60),2),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E44" s="1" t="str">
+        <v>48.02</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>582</v>
+      </c>
+      <c r="D44" s="0" t="n">
+        <v>740</v>
+      </c>
+      <c r="E44" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C44/(D44/60),2),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E45" s="1" t="str">
+        <v>47.19</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>607</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>777</v>
+      </c>
+      <c r="E45" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C45/(D45/60),2),"")</f>
-        <v/>
+        <v>46.87</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>616</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <v>788</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C46/(D46/60),2),"")</f>
+        <v>46.9</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" s="1" t="n">
+        <v>626</v>
+      </c>
+      <c r="D47" s="0" t="n">
+        <v>797</v>
+      </c>
+      <c r="E47" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C47/(D47/60),2),"")</f>
+        <v>47.13</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C48" s="1" t="n">
+        <v>634</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <v>810</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C48/(D48/60),2),"")</f>
+        <v>46.96</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C49" s="1" t="n">
+        <v>639</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <v>820</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C49/(D49/60),2),"")</f>
+        <v>46.76</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add multi-route travel tracker support
</commit_message>
<xml_diff>
--- a/public/data/travel_north_bengal.xlsx
+++ b/public/data/travel_north_bengal.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="123">
   <si>
     <t xml:space="preserve">RailStation</t>
   </si>
@@ -40,6 +40,9 @@
     <t xml:space="preserve">Coordinates</t>
   </si>
   <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bidhannagar</t>
   </si>
   <si>
@@ -85,6 +88,18 @@
     <t xml:space="preserve">22.9567,88.5448</t>
   </si>
   <si>
+    <t xml:space="preserve">Madanpur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayshpur Toll gate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.9603244,88.4590766</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toll</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chakdaha</t>
   </si>
   <si>
@@ -124,6 +139,15 @@
     <t xml:space="preserve">23.4912,88.4590</t>
   </si>
   <si>
+    <t xml:space="preserve">Bethuadahari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sali bamandanga toll plaza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.62909,88.3575211</t>
+  </si>
+  <si>
     <t xml:space="preserve">Palasi</t>
   </si>
   <si>
@@ -136,6 +160,12 @@
     <t xml:space="preserve">23.9312,88.2483</t>
   </si>
   <si>
+    <t xml:space="preserve">Shibpur toll plaza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.1504352,88.1837308</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sagardighi</t>
   </si>
   <si>
@@ -178,6 +208,39 @@
     <t xml:space="preserve">24.8021,87.9171</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">th</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Mile toll plaza</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">24.8223539,87.9644079</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jamirghata</t>
   </si>
   <si>
@@ -229,10 +292,10 @@
     <t xml:space="preserve">25.5891,88.1388</t>
   </si>
   <si>
-    <t xml:space="preserve">Raiganj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.6179,88.1264</t>
+    <t xml:space="preserve">Barai Toll Raiganj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.7145605,87.9594039</t>
   </si>
   <si>
     <t xml:space="preserve">Altapur</t>
@@ -277,10 +340,10 @@
     <t xml:space="preserve">25.8554,87.8540</t>
   </si>
   <si>
-    <t xml:space="preserve">Surajpur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.9214,87.8812</t>
+    <t xml:space="preserve">SurajpurToll plaza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.9335323,87.8405666</t>
   </si>
   <si>
     <t xml:space="preserve">Asurgar</t>
@@ -362,7 +425,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -395,6 +458,13 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -440,7 +510,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -450,6 +520,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -465,7 +539,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -592,7 +666,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.82"/>
@@ -618,73 +692,76 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="B2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>8</v>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">IFERROR(C3/(D3/60),"")</f>
         <v>36</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>11</v>
+      <c r="F3" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>20</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">IFERROR(C4/(D4/60),"")</f>
         <v>36</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>14</v>
+      <c r="F4" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>16</v>
@@ -696,16 +773,16 @@
         <f aca="false">IFERROR(C5/(D5/60),"")</f>
         <v>19.2</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>17</v>
+      <c r="F5" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>59</v>
@@ -717,795 +794,897 @@
         <f aca="false">IFERROR(ROUND(C6/(D6/60),2),"")</f>
         <v>44.25</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>20</v>
+      <c r="F6" s="5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C7/(D7/60),2),"")</f>
-        <v>43.92</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>22</v>
+        <v>44.29</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C8/(D8/60),2),"")</f>
-        <v>46.86</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>24</v>
+        <v>43.92</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="E9" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C9/(D9/60),2),"")</f>
-        <v>48.85</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>26</v>
+        <v>46.86</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E10" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C10/(D10/60),2),"")</f>
-        <v>49.47</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>29</v>
+        <v>48.85</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="E11" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C11/(D11/60),2),"")</f>
-        <v>48.67</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>31</v>
+        <v>49.47</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E12" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C12/(D12/60),2),"")</f>
-        <v>51.84</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>33</v>
+        <v>48.67</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="B13" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>196</v>
+        <v>147</v>
       </c>
       <c r="E13" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C13/(D13/60),2),"")</f>
-        <v>51.12</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>35</v>
+        <v>51.84</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>185</v>
+        <v>145</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>220</v>
+        <v>155</v>
       </c>
       <c r="E14" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C14/(D14/60),2),"")</f>
-        <v>50.45</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>37</v>
+        <v>56.13</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>231</v>
+        <v>167</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>274</v>
+        <v>196</v>
       </c>
       <c r="E15" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C15/(D15/60),2),"")</f>
-        <v>50.58</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>39</v>
+        <v>51.12</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="B16" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>259</v>
+        <v>185</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>305</v>
+        <v>220</v>
       </c>
       <c r="E16" s="1" t="n">
-        <f aca="false">IFERROR(ROUND(C15/(D15/60),2),"")</f>
-        <v>50.58</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>41</v>
+        <f aca="false">IFERROR(ROUND(C16/(D16/60),2),"")</f>
+        <v>50.45</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="0" t="n">
-        <v>330</v>
+        <v>46</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>211</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>241</v>
       </c>
       <c r="E17" s="1" t="n">
-        <f aca="false">IFERROR(ROUND(C16/(D16/60),2),"")</f>
-        <v>50.95</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>43</v>
+        <f aca="false">IFERROR(ROUND(C17/(D17/60),2),"")</f>
+        <v>52.53</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>44</v>
-      </c>
       <c r="B18" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>281</v>
+        <v>231</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>333</v>
+        <v>274</v>
       </c>
       <c r="E18" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C18/(D18/60),2),"")</f>
-        <v>50.63</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>46</v>
+        <v>50.58</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
       <c r="B19" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="0" t="n">
-        <v>340</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="F19" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>259</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>305</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C18/(D18/60),2),"")</f>
+        <v>50.58</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="B20" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="1" t="n">
-        <v>294</v>
+        <v>52</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="E20" s="1" t="n">
-        <f aca="false">IFERROR(ROUND(C20/(D20/60),2),"")</f>
-        <v>50.98</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>51</v>
+        <f aca="false">IFERROR(ROUND(C19/(D19/60),2),"")</f>
+        <v>50.95</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
-        <v>52</v>
+      <c r="A21" s="5" t="s">
+        <v>54</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>318</v>
+        <v>281</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>383</v>
+        <v>333</v>
       </c>
       <c r="E21" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C21/(D21/60),2),"")</f>
-        <v>49.82</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>54</v>
+        <v>50.63</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
       <c r="B22" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" s="0" t="n">
-        <v>400</v>
+        <v>57</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>340</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="4" t="s">
-        <v>56</v>
+      <c r="F22" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>331</v>
+        <v>294</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>410</v>
+        <v>346</v>
       </c>
       <c r="E23" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C23/(D23/60),2),"")</f>
-        <v>48.44</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>58</v>
+        <v>50.98</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>337</v>
+        <v>304</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>415</v>
+        <v>366</v>
       </c>
       <c r="E24" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C24/(D24/60),2),"")</f>
-        <v>48.72</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>60</v>
+        <v>49.84</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="B25" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>349</v>
+        <v>318</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>425</v>
+        <v>383</v>
       </c>
       <c r="E25" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C25/(D25/60),2),"")</f>
-        <v>49.27</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>62</v>
+        <v>49.82</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="1" t="n">
-        <v>357</v>
+        <v>67</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>435</v>
-      </c>
-      <c r="E26" s="1" t="n">
-        <f aca="false">IFERROR(ROUND(C26/(D26/60),2),"")</f>
-        <v>49.24</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>64</v>
+        <v>400</v>
+      </c>
+      <c r="E26" s="1"/>
+      <c r="F26" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="B27" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>385</v>
+        <v>331</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>466</v>
+        <v>410</v>
       </c>
       <c r="E27" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C27/(D27/60),2),"")</f>
-        <v>49.57</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>66</v>
+        <v>48.44</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>400</v>
+        <v>337</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>485</v>
+        <v>415</v>
       </c>
       <c r="E28" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C28/(D28/60),2),"")</f>
-        <v>49.48</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>68</v>
+        <v>48.72</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>423</v>
+        <v>349</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>512</v>
+        <v>425</v>
       </c>
       <c r="E29" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C29/(D29/60),2),"")</f>
-        <v>49.57</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>70</v>
+        <v>49.27</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>423</v>
+        <v>357</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>512</v>
+        <v>435</v>
       </c>
       <c r="E30" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C30/(D30/60),2),"")</f>
-        <v>49.57</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>72</v>
+        <v>49.24</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>426</v>
-      </c>
-      <c r="D31" s="0" t="n">
-        <v>515</v>
+        <v>385</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>466</v>
       </c>
       <c r="E31" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C31/(D31/60),2),"")</f>
-        <v>49.63</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>74</v>
+        <v>49.57</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C32" s="1" t="n">
-        <v>426</v>
+        <v>400</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>520</v>
+        <v>485</v>
       </c>
       <c r="E32" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C32/(D32/60),2),"")</f>
-        <v>49.15</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>76</v>
+        <v>49.48</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D33" s="0" t="n">
-        <v>523</v>
+        <v>81</v>
+      </c>
+      <c r="C33" s="1" t="n">
+        <v>416</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>512</v>
       </c>
       <c r="E33" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C33/(D33/60),2),"")</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>78</v>
+        <v>48.75</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>437</v>
+        <v>423</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>526</v>
+        <v>512</v>
       </c>
       <c r="E34" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C34/(D34/60),2),"")</f>
-        <v>49.85</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>80</v>
+        <v>49.57</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C35" s="1" t="n">
-        <v>442</v>
+        <v>426</v>
       </c>
       <c r="D35" s="1" t="n">
-        <v>536</v>
+        <v>515</v>
       </c>
       <c r="E35" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C35/(D35/60),2),"")</f>
-        <v>49.48</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>82</v>
+        <v>49.63</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>450</v>
+        <v>426</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>545</v>
+        <v>520</v>
       </c>
       <c r="E36" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C36/(D36/60),2),"")</f>
-        <v>49.54</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>84</v>
+        <v>49.15</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D37" s="0" t="n">
-        <v>548</v>
+        <v>89</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>523</v>
       </c>
       <c r="E37" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C37/(D37/60),2),"")</f>
         <v>0</v>
       </c>
-      <c r="F37" s="4" t="s">
-        <v>86</v>
+      <c r="F37" s="5" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D38" s="0" t="n">
-        <v>550</v>
+        <v>91</v>
+      </c>
+      <c r="C38" s="1" t="n">
+        <v>437</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>526</v>
       </c>
       <c r="E38" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C38/(D38/60),2),"")</f>
-        <v>0</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>88</v>
+        <v>49.85</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>467</v>
+        <v>442</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>560</v>
+        <v>536</v>
       </c>
       <c r="E39" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C39/(D39/60),2),"")</f>
-        <v>50.04</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>90</v>
+        <v>49.48</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C40" s="1" t="n">
-        <v>474</v>
+        <v>450</v>
       </c>
       <c r="D40" s="1" t="n">
-        <v>570</v>
+        <v>545</v>
       </c>
       <c r="E40" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C40/(D40/60),2),"")</f>
-        <v>49.89</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>92</v>
+        <v>49.54</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C41" s="1" t="n">
-        <v>481</v>
+        <v>459</v>
       </c>
       <c r="D41" s="1" t="n">
-        <v>600</v>
+        <v>548</v>
       </c>
       <c r="E41" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C41/(D41/60),2),"")</f>
-        <v>48.1</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>94</v>
+        <v>50.26</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C42" s="1" t="n">
-        <v>523</v>
-      </c>
-      <c r="D42" s="0" t="n">
-        <v>653</v>
+      <c r="B42" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>550</v>
       </c>
       <c r="E42" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C42/(D42/60),2),"")</f>
-        <v>48.06</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>96</v>
+        <v>0</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="5" t="s">
-        <v>97</v>
+      <c r="B43" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="C43" s="1" t="n">
-        <v>533</v>
-      </c>
-      <c r="D43" s="0" t="n">
-        <v>666</v>
+        <v>467</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>560</v>
       </c>
       <c r="E43" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C43/(D43/60),2),"")</f>
-        <v>48.02</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>98</v>
+        <v>50.04</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="5" t="s">
-        <v>99</v>
+      <c r="B44" s="1" t="s">
+        <v>103</v>
       </c>
       <c r="C44" s="1" t="n">
-        <v>582</v>
-      </c>
-      <c r="D44" s="0" t="n">
-        <v>740</v>
+        <v>474</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>570</v>
       </c>
       <c r="E44" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C44/(D44/60),2),"")</f>
-        <v>47.19</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>100</v>
+        <v>49.89</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="5" t="s">
-        <v>101</v>
+      <c r="B45" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="C45" s="1" t="n">
-        <v>607</v>
-      </c>
-      <c r="D45" s="0" t="n">
-        <v>777</v>
+        <v>481</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>600</v>
       </c>
       <c r="E45" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C45/(D45/60),2),"")</f>
-        <v>46.87</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>102</v>
+        <v>48.1</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="5" t="s">
-        <v>103</v>
+      <c r="B46" s="4" t="s">
+        <v>107</v>
       </c>
       <c r="C46" s="1" t="n">
-        <v>616</v>
-      </c>
-      <c r="D46" s="0" t="n">
-        <v>788</v>
+        <v>523</v>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>653</v>
       </c>
       <c r="E46" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C46/(D46/60),2),"")</f>
-        <v>46.9</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>104</v>
+        <v>48.06</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="5" t="s">
-        <v>105</v>
+      <c r="B47" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="C47" s="1" t="n">
-        <v>626</v>
-      </c>
-      <c r="D47" s="0" t="n">
-        <v>797</v>
+        <v>533</v>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>666</v>
       </c>
       <c r="E47" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C47/(D47/60),2),"")</f>
-        <v>47.13</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>106</v>
+        <v>48.02</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>107</v>
+      <c r="B48" s="4" t="s">
+        <v>111</v>
       </c>
       <c r="C48" s="1" t="n">
-        <v>634</v>
-      </c>
-      <c r="D48" s="0" t="n">
-        <v>810</v>
+        <v>582</v>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>740</v>
       </c>
       <c r="E48" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C48/(D48/60),2),"")</f>
-        <v>46.96</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>108</v>
+        <v>47.19</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="5" t="s">
-        <v>109</v>
+      <c r="B49" s="4" t="s">
+        <v>113</v>
       </c>
       <c r="C49" s="1" t="n">
-        <v>639</v>
-      </c>
-      <c r="D49" s="0" t="n">
-        <v>820</v>
+        <v>607</v>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>777</v>
       </c>
       <c r="E49" s="1" t="n">
         <f aca="false">IFERROR(ROUND(C49/(D49/60),2),"")</f>
+        <v>46.87</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C50" s="1" t="n">
+        <v>616</v>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>788</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C50/(D50/60),2),"")</f>
+        <v>46.9</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C51" s="1" t="n">
+        <v>626</v>
+      </c>
+      <c r="D51" s="1" t="n">
+        <v>797</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C51/(D51/60),2),"")</f>
+        <v>47.13</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C52" s="1" t="n">
+        <v>634</v>
+      </c>
+      <c r="D52" s="1" t="n">
+        <v>810</v>
+      </c>
+      <c r="E52" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C52/(D52/60),2),"")</f>
+        <v>46.96</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C53" s="1" t="n">
+        <v>639</v>
+      </c>
+      <c r="D53" s="1" t="n">
+        <v>820</v>
+      </c>
+      <c r="E53" s="1" t="n">
+        <f aca="false">IFERROR(ROUND(C53/(D53/60),2),"")</f>
         <v>46.76</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>110</v>
+      <c r="F53" s="7" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>